<commit_message>
Pase el Rosado a Ecuador
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_euro.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_euro.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>687666654</v>
+        <v>701594191</v>
       </c>
     </row>
     <row r="7">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>687666654</v>
+        <v>701594191</v>
       </c>
     </row>
     <row r="8">
@@ -583,7 +583,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>03/11/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>687666654</v>
+        <v>701594191</v>
       </c>
     </row>
     <row r="13"/>
@@ -645,16 +645,16 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>PMP1223601</t>
+          <t>PMP1283592</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>57729245.92</v>
+        <v>103309958.75</v>
       </c>
       <c r="F19" s="10" t="inlineStr"/>
       <c r="G19" s="10" t="inlineStr"/>
       <c r="H19" s="6" t="n">
-        <v>57729245.92</v>
+        <v>103309958.75</v>
       </c>
       <c r="I19" s="11" t="inlineStr"/>
     </row>
@@ -666,16 +666,16 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>PMP1223602</t>
+          <t>PMP1283593</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>30598280.34</v>
+        <v>103299753.4</v>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
       <c r="G20" s="10" t="inlineStr"/>
       <c r="H20" s="6" t="n">
-        <v>30598280.34</v>
+        <v>103299753.4</v>
       </c>
       <c r="I20" s="11" t="inlineStr"/>
     </row>
@@ -687,16 +687,16 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>PMP1225176</t>
+          <t>PMP1286115</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>30598280.34</v>
+        <v>23317782.6</v>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
       <c r="G21" s="10" t="inlineStr"/>
       <c r="H21" s="6" t="n">
-        <v>30598280.34</v>
+        <v>23317782.6</v>
       </c>
       <c r="I21" s="11" t="inlineStr"/>
     </row>
@@ -708,16 +708,16 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>PMP1225177</t>
+          <t>PMP1286453</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>94053401.39</v>
+        <v>25034389.76</v>
       </c>
       <c r="F22" s="10" t="inlineStr"/>
       <c r="G22" s="10" t="inlineStr"/>
       <c r="H22" s="6" t="n">
-        <v>94053401.39</v>
+        <v>25034389.76</v>
       </c>
       <c r="I22" s="11" t="inlineStr"/>
     </row>
@@ -729,16 +729,16 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>PMP1225178</t>
+          <t>PMP1286454</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>34360151.22</v>
+        <v>86198354.58</v>
       </c>
       <c r="F23" s="10" t="inlineStr"/>
       <c r="G23" s="10" t="inlineStr"/>
       <c r="H23" s="6" t="n">
-        <v>34360151.22</v>
+        <v>86198354.58</v>
       </c>
       <c r="I23" s="11" t="inlineStr"/>
     </row>
@@ -750,16 +750,16 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>PMP1225179</t>
+          <t>PMP1286455</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>12229963.96</v>
+        <v>46306658.97</v>
       </c>
       <c r="F24" s="10" t="inlineStr"/>
       <c r="G24" s="10" t="inlineStr"/>
       <c r="H24" s="6" t="n">
-        <v>12229963.96</v>
+        <v>46306658.97</v>
       </c>
       <c r="I24" s="11" t="inlineStr"/>
     </row>
@@ -771,16 +771,16 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>PMP1225180</t>
+          <t>PMP1289255</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>19176448.64</v>
+        <v>60666373.9</v>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
       <c r="G25" s="10" t="inlineStr"/>
       <c r="H25" s="6" t="n">
-        <v>19176448.64</v>
+        <v>60666373.9</v>
       </c>
       <c r="I25" s="11" t="inlineStr"/>
     </row>
@@ -792,16 +792,16 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>PMP1227484</t>
+          <t>PMP1289256</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>8327266.6</v>
+        <v>13452473.7</v>
       </c>
       <c r="F26" s="10" t="inlineStr"/>
       <c r="G26" s="10" t="inlineStr"/>
       <c r="H26" s="6" t="n">
-        <v>8327266.6</v>
+        <v>13452473.7</v>
       </c>
       <c r="I26" s="11" t="inlineStr"/>
     </row>
@@ -813,16 +813,16 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>PMP1227508</t>
+          <t>PMP1289257</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>7984827.6</v>
+        <v>51096639.83</v>
       </c>
       <c r="F27" s="10" t="inlineStr"/>
       <c r="G27" s="10" t="inlineStr"/>
       <c r="H27" s="6" t="n">
-        <v>7984827.6</v>
+        <v>51096639.83</v>
       </c>
       <c r="I27" s="11" t="inlineStr"/>
     </row>
@@ -834,16 +834,16 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>PMP1227531</t>
+          <t>PMP1289258</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>2709787.78</v>
+        <v>2142720.76</v>
       </c>
       <c r="F28" s="10" t="inlineStr"/>
       <c r="G28" s="10" t="inlineStr"/>
       <c r="H28" s="6" t="n">
-        <v>2709787.78</v>
+        <v>2142720.76</v>
       </c>
       <c r="I28" s="11" t="inlineStr"/>
     </row>
@@ -855,16 +855,16 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>PMP1227532</t>
+          <t>PMP1289259</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>17562882.41</v>
+        <v>154694285.44</v>
       </c>
       <c r="F29" s="10" t="inlineStr"/>
       <c r="G29" s="10" t="inlineStr"/>
       <c r="H29" s="6" t="n">
-        <v>17562882.41</v>
+        <v>154694285.44</v>
       </c>
       <c r="I29" s="11" t="inlineStr"/>
     </row>
@@ -876,16 +876,16 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>PMP1227585</t>
+          <t>PMP1292202</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>32215271.66</v>
+        <v>6279096.3</v>
       </c>
       <c r="F30" s="10" t="inlineStr"/>
       <c r="G30" s="10" t="inlineStr"/>
       <c r="H30" s="6" t="n">
-        <v>32215271.66</v>
+        <v>6279096.3</v>
       </c>
       <c r="I30" s="11" t="inlineStr"/>
     </row>
@@ -897,16 +897,16 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>PMP1227644</t>
+          <t>PMP1292208</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>18148048</v>
+        <v>1289757.04</v>
       </c>
       <c r="F31" s="10" t="inlineStr"/>
       <c r="G31" s="10" t="inlineStr"/>
       <c r="H31" s="6" t="n">
-        <v>18148048</v>
+        <v>1289757.04</v>
       </c>
       <c r="I31" s="11" t="inlineStr"/>
     </row>
@@ -918,16 +918,16 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>PMP1230282</t>
+          <t>PMP1292253</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>119818446.6</v>
+        <v>32891959.65</v>
       </c>
       <c r="F32" s="10" t="inlineStr"/>
       <c r="G32" s="10" t="inlineStr"/>
       <c r="H32" s="6" t="n">
-        <v>119818446.6</v>
+        <v>32891959.65</v>
       </c>
       <c r="I32" s="11" t="inlineStr"/>
     </row>
@@ -939,144 +939,212 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>PMP1230283</t>
+          <t>PMP1292726</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>14411572.92</v>
+        <v>8102325.04</v>
       </c>
       <c r="F33" s="10" t="inlineStr"/>
       <c r="G33" s="10" t="inlineStr"/>
       <c r="H33" s="6" t="n">
-        <v>14411572.92</v>
+        <v>8102325.04</v>
       </c>
       <c r="I33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>PMP1230284</t>
+          <t>DE 50434</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>48682759.68</v>
-      </c>
-      <c r="F34" s="10" t="inlineStr"/>
+        <v>-276027</v>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
       <c r="G34" s="10" t="inlineStr"/>
       <c r="H34" s="6" t="n">
-        <v>48682759.68</v>
-      </c>
-      <c r="I34" s="11" t="inlineStr"/>
+        <v>-276027</v>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> DES DE 50434</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>PMP1230285</t>
+          <t>DE 19922</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>33063719.07</v>
-      </c>
-      <c r="F35" s="10" t="inlineStr"/>
-      <c r="G35" s="10" t="inlineStr"/>
+        <v>-55277</v>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H35" s="6" t="n">
-        <v>33063719.07</v>
-      </c>
-      <c r="I35" s="11" t="inlineStr"/>
+        <v>-55277</v>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO CED DE 19922</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>PMP1232380</t>
+          <t>DE 40533</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>78444518.76000001</v>
-      </c>
-      <c r="F36" s="10" t="inlineStr"/>
-      <c r="G36" s="10" t="inlineStr"/>
+        <v>-101818</v>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H36" s="6" t="n">
-        <v>78444518.76000001</v>
-      </c>
-      <c r="I36" s="11" t="inlineStr"/>
+        <v>-101818</v>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO LOB DE 40533</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>PMP1232381</t>
+          <t>DE 55247</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>3261783.44</v>
-      </c>
-      <c r="F37" s="10" t="inlineStr"/>
-      <c r="G37" s="10" t="inlineStr"/>
+        <v>-30454</v>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H37" s="6" t="n">
-        <v>3261783.44</v>
-      </c>
-      <c r="I37" s="11" t="inlineStr"/>
+        <v>-30454</v>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO VEG DE 55247</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>PMP1232382</t>
+          <t>DE 55248</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>24653842.56</v>
-      </c>
-      <c r="F38" s="10" t="inlineStr"/>
-      <c r="G38" s="10" t="inlineStr"/>
+        <v>-87503</v>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H38" s="6" t="n">
-        <v>24653842.56</v>
-      </c>
-      <c r="I38" s="11" t="inlineStr"/>
+        <v>-87503</v>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO VEG DE 55248</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>PMP1232383</t>
+          <t>DE 59457</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>51482393.64</v>
-      </c>
-      <c r="F39" s="10" t="inlineStr"/>
-      <c r="G39" s="10" t="inlineStr"/>
+        <v>-1058911</v>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H39" s="6" t="n">
-        <v>51482393.64</v>
-      </c>
-      <c r="I39" s="11" t="inlineStr"/>
+        <v>-1058911</v>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO LAU DE 59457</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="C40" s="10" t="inlineStr">
@@ -1086,11 +1154,11 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>13154</t>
+          <t>DE 59458</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>-38868</v>
+        <v>-406773</v>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
@@ -1103,11 +1171,11 @@
         </is>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-38868</v>
+        <v>-406773</v>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO TER 13154</t>
+          <t>DESCUENTO LAU DE 59458</t>
         </is>
       </c>
     </row>
@@ -1119,11 +1187,11 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>DE 48462</t>
+          <t>DEC 10778</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>-211513</v>
+        <v>-318584</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -1136,11 +1204,11 @@
         </is>
       </c>
       <c r="H41" s="6" t="n">
-        <v>-211513</v>
+        <v>-318584</v>
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO SAB DE 48462</t>
+          <t>DESCUENTO NUM DEC 10778</t>
         </is>
       </c>
     </row>
@@ -1152,11 +1220,11 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>DE 48487</t>
+          <t>DEC 10779</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>-31124</v>
+        <v>-738452</v>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
@@ -1169,11 +1237,11 @@
         </is>
       </c>
       <c r="H42" s="6" t="n">
-        <v>-31124</v>
+        <v>-738452</v>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO LOB DE 48487</t>
+          <t>DESCUENTO NUM DEC 10779</t>
         </is>
       </c>
     </row>
@@ -1185,11 +1253,11 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>DE 48488</t>
+          <t>DEC 12183</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>-337964</v>
+        <v>-71666</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -1202,11 +1270,11 @@
         </is>
       </c>
       <c r="H43" s="6" t="n">
-        <v>-337964</v>
+        <v>-71666</v>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO LOB DE 48488</t>
+          <t>DESCUENTO MON DEC 12183</t>
         </is>
       </c>
     </row>
@@ -1218,11 +1286,11 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>DE 69379</t>
+          <t>DEC 12766</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>-104706</v>
+        <v>-427050</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
@@ -1235,11 +1303,11 @@
         </is>
       </c>
       <c r="H44" s="6" t="n">
-        <v>-104706</v>
+        <v>-427050</v>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO FLO DE 69379</t>
+          <t>DESCUENTO MIX DEC 12766</t>
         </is>
       </c>
     </row>
@@ -1251,11 +1319,11 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>DE 69380</t>
+          <t>DEC 12767</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>-476562</v>
+        <v>-152019</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -1268,11 +1336,11 @@
         </is>
       </c>
       <c r="H45" s="6" t="n">
-        <v>-476562</v>
+        <v>-152019</v>
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO FLO DE 69380</t>
+          <t>DESCUENTO MIX DEC 12767</t>
         </is>
       </c>
     </row>
@@ -1284,11 +1352,11 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>DE 72961</t>
+          <t>DEC 13340</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>-336853</v>
+        <v>-132594</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
@@ -1301,11 +1369,11 @@
         </is>
       </c>
       <c r="H46" s="6" t="n">
-        <v>-336853</v>
+        <v>-132594</v>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MAY DE 72961</t>
+          <t>DESCUENTO SAL DEC 13340</t>
         </is>
       </c>
     </row>
@@ -1317,11 +1385,11 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>DE 72962</t>
+          <t>DEC 14411</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>-541733</v>
+        <v>-69351</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -1334,11 +1402,11 @@
         </is>
       </c>
       <c r="H47" s="6" t="n">
-        <v>-541733</v>
+        <v>-69351</v>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MAY DE 72962</t>
+          <t>DESCUENTO TER DEC 14411</t>
         </is>
       </c>
     </row>
@@ -1350,11 +1418,11 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>DEC 11372</t>
+          <t>DEC 14899</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>-525803</v>
+        <v>-393979</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
@@ -1367,11 +1435,11 @@
         </is>
       </c>
       <c r="H48" s="6" t="n">
-        <v>-525803</v>
+        <v>-393979</v>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO SAL DEC 11372</t>
+          <t>DESCUENTO MUR DEC 14899</t>
         </is>
       </c>
     </row>
@@ -1383,11 +1451,11 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>DEC 11373</t>
+          <t>DEC 14900</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>-112560</v>
+        <v>-90454</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
@@ -1400,11 +1468,11 @@
         </is>
       </c>
       <c r="H49" s="6" t="n">
-        <v>-112560</v>
+        <v>-90454</v>
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO SAL DEC 11373</t>
+          <t>DESCUENTO MUR DEC 14900</t>
         </is>
       </c>
     </row>
@@ -1416,11 +1484,11 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>DEC 11692</t>
+          <t>DEC 27191</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>-325489</v>
+        <v>-166374</v>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
@@ -1433,11 +1501,11 @@
         </is>
       </c>
       <c r="H50" s="6" t="n">
-        <v>-325489</v>
+        <v>-166374</v>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MIX DEC 11692</t>
+          <t>DESCUENTO ACA DEC 27191</t>
         </is>
       </c>
     </row>
@@ -1449,11 +1517,11 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>DEC 11693</t>
+          <t>DEC 27192</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>-98664</v>
+        <v>-13295</v>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
@@ -1466,11 +1534,11 @@
         </is>
       </c>
       <c r="H51" s="6" t="n">
-        <v>-98664</v>
+        <v>-13295</v>
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MIX DEC 11693</t>
+          <t>DESCUENTO ACA DEC 27192</t>
         </is>
       </c>
     </row>
@@ -1482,11 +1550,11 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>DEC 13155</t>
+          <t>DEC 28349</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>-151030</v>
+        <v>-5333</v>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
@@ -1499,11 +1567,11 @@
         </is>
       </c>
       <c r="H52" s="6" t="n">
-        <v>-151030</v>
+        <v>-5333</v>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO TER DEC 13155</t>
+          <t>DESCUENTO ITA DEC 28349</t>
         </is>
       </c>
     </row>
@@ -1515,11 +1583,11 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>DEC 13898</t>
+          <t>DEC 28350</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>-96982</v>
+        <v>-63180</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
@@ -1532,11 +1600,11 @@
         </is>
       </c>
       <c r="H53" s="6" t="n">
-        <v>-96982</v>
+        <v>-63180</v>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MUR DEC 13898</t>
+          <t>DESCUENTO ITA DEC 28350</t>
         </is>
       </c>
     </row>
@@ -1548,11 +1616,11 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>DEC 13899</t>
+          <t>DEC 41222</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>-37834</v>
+        <v>-624783</v>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
@@ -1565,11 +1633,11 @@
         </is>
       </c>
       <c r="H54" s="6" t="n">
-        <v>-37834</v>
+        <v>-624783</v>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO MUR DEC 13899</t>
+          <t>DESCUENTO BEL DEC 41222</t>
         </is>
       </c>
     </row>
@@ -1581,11 +1649,11 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>DEC 19801</t>
+          <t>DEC 41223</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>-71906</v>
+        <v>-88054</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -1598,11 +1666,11 @@
         </is>
       </c>
       <c r="H55" s="6" t="n">
-        <v>-71906</v>
+        <v>-88054</v>
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO CED DEC 19801</t>
+          <t>DESCUENTO BEL DEC 41223</t>
         </is>
       </c>
     </row>
@@ -1614,11 +1682,11 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>DEC 19802</t>
+          <t>DEC 50261</t>
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>-222861</v>
+        <v>-4340859</v>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
@@ -1631,11 +1699,11 @@
         </is>
       </c>
       <c r="H56" s="6" t="n">
-        <v>-222861</v>
+        <v>-4340859</v>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO CED DEC 19802</t>
+          <t>DESCUENTO SAB DEC 50261</t>
         </is>
       </c>
     </row>
@@ -1647,11 +1715,11 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>DEC 24237</t>
+          <t>DEC 50261</t>
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>-139435</v>
+        <v>-486838</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -1664,11 +1732,11 @@
         </is>
       </c>
       <c r="H57" s="6" t="n">
-        <v>-139435</v>
+        <v>-486838</v>
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO LLA DEC 24237</t>
+          <t>DESCUENTO SAB DEC 50261</t>
         </is>
       </c>
     </row>
@@ -1680,11 +1748,11 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>DEC 24238</t>
+          <t>DEC 50589</t>
         </is>
       </c>
       <c r="E58" s="6" t="n">
-        <v>-239141</v>
+        <v>-219844</v>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
@@ -1697,11 +1765,11 @@
         </is>
       </c>
       <c r="H58" s="6" t="n">
-        <v>-239141</v>
+        <v>-219844</v>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO LLA DEC 24238</t>
+          <t>DESCUENTO SAB DEC 50589</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1781,11 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>DEC 25124</t>
+          <t>DEC 50590</t>
         </is>
       </c>
       <c r="E59" s="6" t="n">
-        <v>-174033</v>
+        <v>-623109</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
@@ -1730,11 +1798,11 @@
         </is>
       </c>
       <c r="H59" s="6" t="n">
-        <v>-174033</v>
+        <v>-623109</v>
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ACA DEC 25124</t>
+          <t>DESCUENTO SAB DEC 50590</t>
         </is>
       </c>
     </row>
@@ -1746,11 +1814,11 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>DEC 25125</t>
+          <t>DEC 55597</t>
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>-36033</v>
+        <v>-222657</v>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
@@ -1763,11 +1831,11 @@
         </is>
       </c>
       <c r="H60" s="6" t="n">
-        <v>-36033</v>
+        <v>-222657</v>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ACA DEC 25125</t>
+          <t>DESCUENTO VEG DEC 55597</t>
         </is>
       </c>
     </row>
@@ -1779,11 +1847,11 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>DEC 27272</t>
+          <t>DEC 55598</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>-128068</v>
+        <v>-148012</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -1796,11 +1864,11 @@
         </is>
       </c>
       <c r="H61" s="6" t="n">
-        <v>-128068</v>
+        <v>-148012</v>
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ITA DEC 27272</t>
+          <t>DESCUENTO VEG DEC 55598</t>
         </is>
       </c>
     </row>
@@ -1812,11 +1880,11 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>DEC 27273</t>
+          <t>DEC 57536</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>-43522</v>
+        <v>-35833</v>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
@@ -1829,11 +1897,11 @@
         </is>
       </c>
       <c r="H62" s="6" t="n">
-        <v>-43522</v>
+        <v>-35833</v>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ITA DEC 27273</t>
+          <t>DESCUENTO GUA DEC 57536</t>
         </is>
       </c>
     </row>
@@ -1845,11 +1913,11 @@
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>DEC 48461</t>
+          <t>DEC 57537</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>-156305</v>
+        <v>-322534</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -1862,11 +1930,11 @@
         </is>
       </c>
       <c r="H63" s="6" t="n">
-        <v>-156305</v>
+        <v>-322534</v>
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO SAB DEC 48461</t>
+          <t>DESCUENTO GUA DEC 57537</t>
         </is>
       </c>
     </row>
@@ -1878,11 +1946,11 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>DEC 53645</t>
+          <t>DEC 71005</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>-34392</v>
+        <v>-1013389</v>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
@@ -1895,11 +1963,11 @@
         </is>
       </c>
       <c r="H64" s="6" t="n">
-        <v>-34392</v>
+        <v>-1013389</v>
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO VEG DEC 53645</t>
+          <t>DESCUENTO FLO DEC 71005</t>
         </is>
       </c>
     </row>
@@ -1911,11 +1979,11 @@
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>DEC 53646</t>
+          <t>DEC 71006</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>-284304</v>
+        <v>-192818</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -1928,11 +1996,11 @@
         </is>
       </c>
       <c r="H65" s="6" t="n">
-        <v>-284304</v>
+        <v>-192818</v>
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO VEG DEC 53646</t>
+          <t>DESCUENTO FLO DEC 71006</t>
         </is>
       </c>
     </row>
@@ -1944,11 +2012,11 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>DEC 55933</t>
+          <t>DEC 7389</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>-317598</v>
+        <v>-234580</v>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
@@ -1961,11 +2029,11 @@
         </is>
       </c>
       <c r="H66" s="6" t="n">
-        <v>-317598</v>
+        <v>-234580</v>
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO GUA DEC 55933</t>
+          <t>DESCUENTO ROS DEC 7389</t>
         </is>
       </c>
     </row>
@@ -1977,11 +2045,11 @@
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>DEC 55934</t>
+          <t>DEC 7390</t>
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>-131736</v>
+        <v>-55459</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -1994,11 +2062,11 @@
         </is>
       </c>
       <c r="H67" s="6" t="n">
-        <v>-131736</v>
+        <v>-55459</v>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO GUA DEC 55934</t>
+          <t>DESCUENTO ROS DEC 7390</t>
         </is>
       </c>
     </row>
@@ -2010,11 +2078,11 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>DEC 6808</t>
+          <t>DEC 74875</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>-364123</v>
+        <v>-211524</v>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
@@ -2027,11 +2095,11 @@
         </is>
       </c>
       <c r="H68" s="6" t="n">
-        <v>-364123</v>
+        <v>-211524</v>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ROS DEC 6808</t>
+          <t>DESCUENTO MAY DEC 74875</t>
         </is>
       </c>
     </row>
@@ -2043,11 +2111,11 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>DEC 6809</t>
+          <t>DEC 74876</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>-114728</v>
+        <v>-191186</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -2060,11 +2128,11 @@
         </is>
       </c>
       <c r="H69" s="6" t="n">
-        <v>-114728</v>
+        <v>-191186</v>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO ROS DEC 6809</t>
+          <t>DESCUENTO MAY DEC 74876</t>
         </is>
       </c>
     </row>
@@ -2076,11 +2144,11 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>DEC 7317</t>
+          <t>DEC 7819</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>-88412</v>
+        <v>-280549</v>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
@@ -2093,11 +2161,11 @@
         </is>
       </c>
       <c r="H70" s="6" t="n">
-        <v>-88412</v>
+        <v>-280549</v>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO CAR DEC 7317</t>
+          <t>DESCUENTO CAR DEC 7819</t>
         </is>
       </c>
     </row>
@@ -2109,11 +2177,11 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>DEC 7318</t>
+          <t>DEC 7820</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>-84338</v>
+        <v>-30515</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -2126,11 +2194,11 @@
         </is>
       </c>
       <c r="H71" s="6" t="n">
-        <v>-84338</v>
+        <v>-30515</v>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO CAR DEC 7318</t>
+          <t>DESCUENTO CAR DEC 7820</t>
         </is>
       </c>
     </row>
@@ -2142,11 +2210,11 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>DEC 79615</t>
+          <t>DEC 7821</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>-53026</v>
+        <v>-21910</v>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
@@ -2159,11 +2227,11 @@
         </is>
       </c>
       <c r="H72" s="6" t="n">
-        <v>-53026</v>
+        <v>-21910</v>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO FRO DEC 79615</t>
+          <t>DESCUENTO CAR DEC 7821</t>
         </is>
       </c>
     </row>
@@ -2175,11 +2243,11 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>DEC 79616</t>
+          <t>DEC 81904</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>-72370</v>
+        <v>-193712</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -2192,11 +2260,11 @@
         </is>
       </c>
       <c r="H73" s="6" t="n">
-        <v>-72370</v>
+        <v>-193712</v>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO FRO DEC 79616</t>
+          <t>DESCUENTO FRO DEC 81904</t>
         </is>
       </c>
     </row>
@@ -2208,15 +2276,15 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>PMP1223601</t>
+          <t>DEC 81905</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>42913732.92</v>
+        <v>-149173</v>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
@@ -2225,11 +2293,11 @@
         </is>
       </c>
       <c r="H74" s="6" t="n">
-        <v>42913732.92</v>
+        <v>-149173</v>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1223601</t>
+          <t>DESCUENTO FRO DEC 81905</t>
         </is>
       </c>
     </row>
@@ -2241,15 +2309,15 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>PMP1225176</t>
+          <t>DEV 13341</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>163627.3399999999</v>
+        <v>-172691</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="G75" s="10" t="inlineStr">
@@ -2258,11 +2326,11 @@
         </is>
       </c>
       <c r="H75" s="6" t="n">
-        <v>163627.3399999999</v>
+        <v>-172691</v>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1225176</t>
+          <t>DESCUENTO SAL DEV 13341</t>
         </is>
       </c>
     </row>
@@ -2274,15 +2342,15 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>PMP1225178</t>
+          <t>DEV 14410</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>121217.2199999988</v>
+        <v>-161295</v>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
@@ -2291,11 +2359,11 @@
         </is>
       </c>
       <c r="H76" s="6" t="n">
-        <v>121217.2199999988</v>
+        <v>-161295</v>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1225178</t>
+          <t>DESCUENTO TER DEV 14410</t>
         </is>
       </c>
     </row>
@@ -2307,11 +2375,11 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>PMP1227508</t>
+          <t>PMP1286454</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>229431.5999999996</v>
+        <v>476112.5799999982</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -2324,11 +2392,11 @@
         </is>
       </c>
       <c r="H77" s="6" t="n">
-        <v>229431.5999999996</v>
+        <v>476112.5799999982</v>
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1227508</t>
+          <t>Myr Vlr Pagado PMP1286454</t>
         </is>
       </c>
     </row>
@@ -2340,11 +2408,11 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1227585</t>
+          <t>PMP1286455</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>295304.6600000001</v>
+        <v>219219.9699999988</v>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
@@ -2357,11 +2425,11 @@
         </is>
       </c>
       <c r="H78" s="6" t="n">
-        <v>295304.6600000001</v>
+        <v>219219.9699999988</v>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1227585</t>
+          <t>Myr Vlr Pagado PMP1286455</t>
         </is>
       </c>
     </row>
@@ -2373,11 +2441,11 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>PMP1230284</t>
+          <t>PMP1289255</t>
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>298845.6799999997</v>
+        <v>613271.8999999985</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -2390,11 +2458,11 @@
         </is>
       </c>
       <c r="H79" s="6" t="n">
-        <v>298845.6799999997</v>
+        <v>613271.8999999985</v>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1230284</t>
+          <t>Myr Vlr Pagado PMP1289255</t>
         </is>
       </c>
     </row>
@@ -2406,11 +2474,11 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>PMP1230285</t>
+          <t>PMP1289256</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>732071.0700000003</v>
+        <v>239040.6999999993</v>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
@@ -2423,11 +2491,11 @@
         </is>
       </c>
       <c r="H80" s="6" t="n">
-        <v>732071.0700000003</v>
+        <v>239040.6999999993</v>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1230285</t>
+          <t>Myr Vlr Pagado PMP1289256</t>
         </is>
       </c>
     </row>
@@ -2439,11 +2507,11 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>PMP1232383</t>
+          <t>PMP1289257</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>908074.6400000006</v>
+        <v>86963.82999999821</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -2456,11 +2524,11 @@
         </is>
       </c>
       <c r="H81" s="6" t="n">
-        <v>908074.6400000006</v>
+        <v>86963.82999999821</v>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1232383</t>
+          <t>Myr Vlr Pagado PMP1289257</t>
         </is>
       </c>
     </row>
@@ -2472,26 +2540,59 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
+          <t>PMP1292253</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>173165.6499999985</v>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>Myr Vlr Pagado</t>
+        </is>
+      </c>
+      <c r="G82" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="n">
+        <v>173165.6499999985</v>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>Myr Vlr Pagado PMP1292253</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>Descuento Cliente</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
           <t>MENORES VALORES</t>
         </is>
       </c>
-      <c r="E82" s="6" t="n">
-        <v>-82.60000000055879</v>
-      </c>
-      <c r="F82" s="10" t="inlineStr">
+      <c r="E83" s="6" t="n">
+        <v>146.0900000063702</v>
+      </c>
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>
       </c>
-      <c r="G82" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H82" s="6" t="n">
-        <v>-82.60000000055879</v>
-      </c>
-      <c r="I82" s="11" t="inlineStr">
+      <c r="G83" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="n">
+        <v>146.0900000063702</v>
+      </c>
+      <c r="I83" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>
@@ -2508,7 +2609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2561,22 +2662,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DE 72962</t>
+          <t>DEC 50261</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>541,733</t>
+          <t>4,340,859</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2586,12 +2687,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>541,733</t>
+          <t>4,340,859</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>-541,733</t>
+          <t>-4,340,859</t>
         </is>
       </c>
     </row>
@@ -2603,22 +2704,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DE 72961</t>
+          <t>DEC 50590</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>336,853</t>
+          <t>623,109</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2628,12 +2729,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>336,853</t>
+          <t>623,109</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-336,853</t>
+          <t>-623,109</t>
         </is>
       </c>
     </row>
@@ -2645,22 +2746,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DEC 11372</t>
+          <t>DEC 50261</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>525,803</t>
+          <t>486,838</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2670,12 +2771,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>525,803</t>
+          <t>486,838</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>-525,803</t>
+          <t>-486,838</t>
         </is>
       </c>
     </row>
@@ -2687,22 +2788,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DEC 11373</t>
+          <t>DEC 50589</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>112,560</t>
+          <t>219,844</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2712,12 +2813,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>112,560</t>
+          <t>219,844</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>-112,560</t>
+          <t>-219,844</t>
         </is>
       </c>
     </row>
@@ -2729,22 +2830,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>LAU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DE 69380</t>
+          <t>DE 59457</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>476,562</t>
+          <t>1,058,911</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2754,12 +2855,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>476,562</t>
+          <t>1,058,911</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-476,562</t>
+          <t>-1,058,911</t>
         </is>
       </c>
     </row>
@@ -2771,22 +2872,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>LAU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DE 69379</t>
+          <t>DE 59458</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>104,706</t>
+          <t>406,773</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2796,12 +2897,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>104,706</t>
+          <t>406,773</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-104,706</t>
+          <t>-406,773</t>
         </is>
       </c>
     </row>
@@ -2813,22 +2914,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ROS</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DEC 6808</t>
+          <t>DEC 71005</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>364,123</t>
+          <t>1,013,389</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2838,12 +2939,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>364,123</t>
+          <t>1,013,389</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>-364,123</t>
+          <t>-1,013,389</t>
         </is>
       </c>
     </row>
@@ -2855,22 +2956,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ROS</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DEC 6809</t>
+          <t>DEC 71006</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>114,728</t>
+          <t>192,818</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2880,12 +2981,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>114,728</t>
+          <t>192,818</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>-114,728</t>
+          <t>-192,818</t>
         </is>
       </c>
     </row>
@@ -2897,22 +2998,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LOB</t>
+          <t>NUM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DE 48488</t>
+          <t>DEC 10779</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>337,964</t>
+          <t>738,452</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2922,12 +3023,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>337,964</t>
+          <t>738,452</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-337,964</t>
+          <t>-738,452</t>
         </is>
       </c>
     </row>
@@ -2939,22 +3040,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LOB</t>
+          <t>NUM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DE 48487</t>
+          <t>DEC 10778</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>31,124</t>
+          <t>318,584</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2964,12 +3065,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>31,124</t>
+          <t>318,584</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>-31,124</t>
+          <t>-318,584</t>
         </is>
       </c>
     </row>
@@ -2981,22 +3082,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MIX</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DEC 11692</t>
+          <t>DEC 41222</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>325,489</t>
+          <t>624,783</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -3006,12 +3107,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>325,489</t>
+          <t>624,783</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>-325,489</t>
+          <t>-624,783</t>
         </is>
       </c>
     </row>
@@ -3023,22 +3124,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MIX</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DEC 11693</t>
+          <t>DEC 41223</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>98,664</t>
+          <t>88,054</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3048,12 +3149,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>98,664</t>
+          <t>88,054</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>-98,664</t>
+          <t>-88,054</t>
         </is>
       </c>
     </row>
@@ -3065,22 +3166,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GUA</t>
+          <t>MIX</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DEC 55933</t>
+          <t>DEC 12766</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>317,598</t>
+          <t>427,050</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3090,12 +3191,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>317,598</t>
+          <t>427,050</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>-317,598</t>
+          <t>-427,050</t>
         </is>
       </c>
     </row>
@@ -3107,22 +3208,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GUA</t>
+          <t>MIX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DEC 55934</t>
+          <t>DEC 12767</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>131,736</t>
+          <t>152,019</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3132,12 +3233,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>131,736</t>
+          <t>152,019</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>-131,736</t>
+          <t>-152,019</t>
         </is>
       </c>
     </row>
@@ -3149,22 +3250,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VEG</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DEC 53646</t>
+          <t>DEC 14899</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>284,304</t>
+          <t>393,979</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3174,12 +3275,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>284,304</t>
+          <t>393,979</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>-284,304</t>
+          <t>-393,979</t>
         </is>
       </c>
     </row>
@@ -3191,22 +3292,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VEG</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DEC 53645</t>
+          <t>DEC 14900</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>34,392</t>
+          <t>90,454</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3216,12 +3317,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>34,392</t>
+          <t>90,454</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>-34,392</t>
+          <t>-90,454</t>
         </is>
       </c>
     </row>
@@ -3233,22 +3334,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LLA</t>
+          <t>GUA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DEC 24238</t>
+          <t>DEC 57537</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>239,141</t>
+          <t>322,534</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3258,12 +3359,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>239,141</t>
+          <t>322,534</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>-239,141</t>
+          <t>-322,534</t>
         </is>
       </c>
     </row>
@@ -3275,22 +3376,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LLA</t>
+          <t>GUA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DEC 24237</t>
+          <t>DEC 57536</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>139,435</t>
+          <t>35,833</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3300,12 +3401,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>139,435</t>
+          <t>35,833</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>-139,435</t>
+          <t>-35,833</t>
         </is>
       </c>
     </row>
@@ -3317,22 +3418,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DEC 19802</t>
+          <t>DEC 7819</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>222,861</t>
+          <t>280,549</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3342,12 +3443,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>222,861</t>
+          <t>280,549</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>-222,861</t>
+          <t>-280,549</t>
         </is>
       </c>
     </row>
@@ -3359,22 +3460,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DEC 19801</t>
+          <t>DEC 7820</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>71,906</t>
+          <t>30,515</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3384,12 +3485,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>71,906</t>
+          <t>30,515</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-71,906</t>
+          <t>-30,515</t>
         </is>
       </c>
     </row>
@@ -3401,22 +3502,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SAB</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DE 48462</t>
+          <t>DEC 7821</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>211,513</t>
+          <t>21,910</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3426,12 +3527,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>211,513</t>
+          <t>21,910</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-211,513</t>
+          <t>-21,910</t>
         </is>
       </c>
     </row>
@@ -3443,22 +3544,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SAB</t>
+          <t>DES</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DEC 48461</t>
+          <t>DE 50434</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>156,305</t>
+          <t>276,027</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3468,12 +3569,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>156,305</t>
+          <t>276,027</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-156,305</t>
+          <t>-276,027</t>
         </is>
       </c>
     </row>
@@ -3485,22 +3586,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ROS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DEC 25124</t>
+          <t>DEC 7389</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>174,033</t>
+          <t>234,580</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3510,12 +3611,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>174,033</t>
+          <t>234,580</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>-174,033</t>
+          <t>-234,580</t>
         </is>
       </c>
     </row>
@@ -3527,22 +3628,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ROS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DEC 25125</t>
+          <t>DEC 7390</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>36,033</t>
+          <t>55,459</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3552,12 +3653,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>36,033</t>
+          <t>55,459</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>-36,033</t>
+          <t>-55,459</t>
         </is>
       </c>
     </row>
@@ -3569,22 +3670,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>VEG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DEC 13155</t>
+          <t>DEC 55597</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>151,030</t>
+          <t>222,657</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3594,12 +3695,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>151,030</t>
+          <t>222,657</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>-151,030</t>
+          <t>-222,657</t>
         </is>
       </c>
     </row>
@@ -3611,22 +3712,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>VEG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>13154</t>
+          <t>DEC 55598</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>38,868</t>
+          <t>148,012</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3636,12 +3737,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>38,868</t>
+          <t>148,012</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>-38,868</t>
+          <t>-148,012</t>
         </is>
       </c>
     </row>
@@ -3653,22 +3754,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>VEG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DEC 27272</t>
+          <t>DE 55248</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>128,068</t>
+          <t>87,503</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3678,12 +3779,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>128,068</t>
+          <t>87,503</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>-128,068</t>
+          <t>-87,503</t>
         </is>
       </c>
     </row>
@@ -3695,22 +3796,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>VEG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DEC 27273</t>
+          <t>DE 55247</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>43,522</t>
+          <t>30,454</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3720,12 +3821,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>43,522</t>
+          <t>30,454</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>-43,522</t>
+          <t>-30,454</t>
         </is>
       </c>
     </row>
@@ -3737,22 +3838,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MAY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DEC 13898</t>
+          <t>DEC 74875</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>96,982</t>
+          <t>211,524</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3762,12 +3863,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>96,982</t>
+          <t>211,524</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>-96,982</t>
+          <t>-211,524</t>
         </is>
       </c>
     </row>
@@ -3779,22 +3880,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MAY</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DEC 13899</t>
+          <t>DEC 74876</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>37,834</t>
+          <t>191,186</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3804,12 +3905,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>37,834</t>
+          <t>191,186</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>-37,834</t>
+          <t>-191,186</t>
         </is>
       </c>
     </row>
@@ -3821,22 +3922,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>FRO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DEC 7317</t>
+          <t>DEC 81904</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>88,412</t>
+          <t>193,712</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3846,12 +3947,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>88,412</t>
+          <t>193,712</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>-88,412</t>
+          <t>-193,712</t>
         </is>
       </c>
     </row>
@@ -3863,22 +3964,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>FRO</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DEC 7318</t>
+          <t>DEC 81905</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>84,338</t>
+          <t>149,173</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3888,12 +3989,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>84,338</t>
+          <t>149,173</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>-84,338</t>
+          <t>-149,173</t>
         </is>
       </c>
     </row>
@@ -3905,22 +4006,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>FRO</t>
+          <t>SAL</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>DEC 79616</t>
+          <t>DEV 13341</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>72,370</t>
+          <t>172,691</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3930,12 +4031,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>72,370</t>
+          <t>172,691</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>-72,370</t>
+          <t>-172,691</t>
         </is>
       </c>
     </row>
@@ -3947,22 +4048,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FRO</t>
+          <t>SAL</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>DEC 79615</t>
+          <t>DEC 13340</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>53,026</t>
+          <t>132,594</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3972,12 +4073,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>53,026</t>
+          <t>132,594</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>-53,026</t>
+          <t>-132,594</t>
         </is>
       </c>
     </row>
@@ -3989,22 +4090,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PMP 1227531</t>
+          <t>DEC 27191</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2,709,788</t>
+          <t>166,374</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4014,12 +4115,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2,709,788</t>
+          <t>166,374</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2,709,788</t>
+          <t>-166,374</t>
         </is>
       </c>
     </row>
@@ -4031,22 +4132,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PMP 1232381</t>
+          <t>DEC 27192</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>3,261,784</t>
+          <t>13,295</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4056,12 +4157,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>3,261,784</t>
+          <t>13,295</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>3,261,784</t>
+          <t>-13,295</t>
         </is>
       </c>
     </row>
@@ -4073,22 +4174,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PMP 1227508</t>
+          <t>DEV 14410</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>7,984,835</t>
+          <t>161,295</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4098,12 +4199,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>7,984,835</t>
+          <t>161,295</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>7,755,396</t>
+          <t>-161,295</t>
         </is>
       </c>
     </row>
@@ -4115,22 +4216,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PMP 1227484</t>
+          <t>DEC 14411</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>8,327,266</t>
+          <t>69,351</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4140,12 +4241,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>8,327,266</t>
+          <t>69,351</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>8,327,266</t>
+          <t>-69,351</t>
         </is>
       </c>
     </row>
@@ -4157,22 +4258,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>LOB</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PMP 1225179</t>
+          <t>DE 40533</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>12,229,966</t>
+          <t>101,818</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4182,12 +4283,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>12,229,966</t>
+          <t>101,818</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>12,229,966</t>
+          <t>-101,818</t>
         </is>
       </c>
     </row>
@@ -4199,22 +4300,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PMP 1230283</t>
+          <t>DEC 12183</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>14,411,575</t>
+          <t>71,666</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4224,12 +4325,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>14,411,575</t>
+          <t>71,666</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>14,411,575</t>
+          <t>-71,666</t>
         </is>
       </c>
     </row>
@@ -4241,22 +4342,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PMP 1223601</t>
+          <t>DEC 28350</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>57,729,246</t>
+          <t>63,180</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4266,12 +4367,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>57,729,246</t>
+          <t>63,180</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>14,815,513</t>
+          <t>-63,180</t>
         </is>
       </c>
     </row>
@@ -4283,22 +4384,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CED</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PMP 1227532</t>
+          <t>DEC 28349</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>17,562,909</t>
+          <t>5,333</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4308,12 +4409,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>17,562,909</t>
+          <t>5,333</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>17,562,909</t>
+          <t>-5,333</t>
         </is>
       </c>
     </row>
@@ -4330,17 +4431,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PMP 12276442</t>
+          <t>DE 19922</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>18,148,045</t>
+          <t>55,277</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4350,12 +4451,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>18,148,045</t>
+          <t>55,277</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>18,148,045</t>
+          <t>-55,277</t>
         </is>
       </c>
     </row>
@@ -4372,17 +4473,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PMP 1225180</t>
+          <t>PMP 1292208</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>19,176,446</t>
+          <t>1,289,757</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4392,12 +4493,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>19,176,446</t>
+          <t>1,289,757</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19,176,446</t>
+          <t>1,289,757</t>
         </is>
       </c>
     </row>
@@ -4414,17 +4515,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PM 1232382</t>
+          <t>PMP 1289258</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>24,653,843</t>
+          <t>2,142,721</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4434,12 +4535,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>24,653,843</t>
+          <t>2,142,721</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24,653,843</t>
+          <t>2,142,721</t>
         </is>
       </c>
     </row>
@@ -4456,17 +4557,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PMP 1225176</t>
+          <t>PMP 1292202</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>30,598,280</t>
+          <t>6,279,095</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4476,12 +4577,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>30,598,280</t>
+          <t>6,279,095</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>30,434,653</t>
+          <t>6,279,095</t>
         </is>
       </c>
     </row>
@@ -4498,17 +4599,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PMP 1223602</t>
+          <t>PMP 1292726</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>30,598,280</t>
+          <t>8,102,323</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4518,12 +4619,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>30,598,280</t>
+          <t>8,102,323</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>30,598,280</t>
+          <t>8,102,323</t>
         </is>
       </c>
     </row>
@@ -4540,17 +4641,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PMP 1227585</t>
+          <t>PMP 1289256</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>32,215,273</t>
+          <t>13,452,473</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4560,12 +4661,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>32,215,273</t>
+          <t>13,452,473</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>31,919,967</t>
+          <t>13,213,433</t>
         </is>
       </c>
     </row>
@@ -4582,17 +4683,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PMP 1230285</t>
+          <t>PMP 1286115</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>33,063,736</t>
+          <t>23,317,782</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4602,12 +4703,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>33,063,736</t>
+          <t>23,317,782</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>32,331,648</t>
+          <t>23,317,782</t>
         </is>
       </c>
     </row>
@@ -4624,17 +4725,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PMP 1225178</t>
+          <t>PMP 1286453</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>34,360,252</t>
+          <t>25,034,390</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4644,12 +4745,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>34,360,252</t>
+          <t>25,034,390</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>34,238,934</t>
+          <t>25,034,390</t>
         </is>
       </c>
     </row>
@@ -4666,17 +4767,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PMP 1230284</t>
+          <t>PMP 1283592</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>48,682,832</t>
+          <t>30,442,266</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4686,12 +4787,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>48,682,832</t>
+          <t>103,309,816</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>48,383,914</t>
+          <t>103,309,816</t>
         </is>
       </c>
     </row>
@@ -4708,17 +4809,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PMP 1232383</t>
+          <t>PMP 1292253</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>51,482,483</t>
+          <t>32,891,970</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4728,12 +4829,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>51,482,483</t>
+          <t>32,891,970</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>50,574,319</t>
+          <t>32,718,794</t>
         </is>
       </c>
     </row>
@@ -4750,17 +4851,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PM 1232380</t>
+          <t>PMP 1286455</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>78,444,570</t>
+          <t>46,306,560</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4770,12 +4871,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>78,444,570</t>
+          <t>46,306,560</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>78,444,570</t>
+          <t>46,087,439</t>
         </is>
       </c>
     </row>
@@ -4792,17 +4893,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PMP 1225177</t>
+          <t>PMP 1289257</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>94,053,410</t>
+          <t>51,096,546</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4812,12 +4913,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>94,053,410</t>
+          <t>51,096,546</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>94,053,410</t>
+          <t>51,009,676</t>
         </is>
       </c>
     </row>
@@ -4834,17 +4935,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PMP 1230282</t>
+          <t>PMP 1289255</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>INV 30 MAYO</t>
+          <t>INV II 31 OCT</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>116,374,948</t>
+          <t>60,666,438</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4854,12 +4955,138 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>119,818,444</t>
+          <t>60,666,438</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>119,818,444</t>
+          <t>60,053,102</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>CED</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PMP 1286454</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>INV II 31 OCT</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>86,198,508</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>86,198,508</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>85,722,242</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CED</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PMP 1283593</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>INV II 31 OCT</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>103,113,605</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>103,299,753</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>103,299,753</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>CED</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PMP 1289259</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>INV II 31 OCT</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>153,763,546</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>154,694,286</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>154,694,286</t>
         </is>
       </c>
     </row>

</xml_diff>